<commit_message>
Lista de visitas: pestaña de consultoras dentales
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012MTkCLosapjNbCkUbLxrE1
</commit_message>
<xml_diff>
--- a/reports/Lista de visitas Valencia.xlsx
+++ b/reports/Lista de visitas Valencia.xlsx
@@ -8,16 +8,18 @@
   </bookViews>
   <sheets>
     <sheet name="Cómo usarla" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Empresas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Consultoras" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Escuelas y cámaras" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="FP y academias" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Consultoras dentales" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Empresas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Consultoras" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Escuelas y cámaras" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FP y academias" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Empresas'!$A$1:$P$49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Consultoras'!$A$1:$O$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Escuelas y cámaras'!$A$1:$O$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'FP y academias'!$A$1:$O$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Consultoras dentales'!$A$1:$J$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Empresas'!$A$1:$P$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Consultoras'!$A$1:$O$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Escuelas y cámaras'!$A$1:$O$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'FP y academias'!$A$1:$O$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,6 +592,634 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Prioridad</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Consultora</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Dónde</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Qué hace (según su web o el buscador)</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Persona pública</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Por qué encaja</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Próximo paso / resultado</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Metodoclinic</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Valencia</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Consultoría estratégica dental: operaciones, coaching, gestión y liderazgo. Tiene un curso online 'Experto en ventas y comunicación' para clínicas dentales.</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr"/>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>https://metodoclinic.com/</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Está en Valencia y ya forma en ventas a equipos de clínica: se puede visitar.</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>Por llamar</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr"/>
+      <c r="J2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Brains and Teeth Consulting Group</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Valencia</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Consultoría dental en Valencia con enfoque ético y estratégico.</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr"/>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>https://brainsandteethconsultinggroup.es/</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Está en Valencia; confirmar si forma a coordinadoras.</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Por llamar</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr"/>
+      <c r="J3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Plan Synergia</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Valencia</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Equipo de dentistas y consultores en gestión estratégica de clínicas dentales.</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>(buscar web)</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Está en Valencia; confirmar si forma a coordinadoras.</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Por llamar</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr"/>
+      <c r="J4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Fran Caro Consultores</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Sin confirmar (formado en la Universidad de Valencia)</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Consultoría dental desde 2013 con formaciones a medida en gestión, entrenamiento comercial y área financiera. Dirige el Máster en Gestión de Clínica Dental de La Salle (Madrid). Cofundador de Global Talent Clinics.</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Fran Caro, fundador y CEO (web propia y prensa del sector)</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>https://www.francaro.es/</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Hace 'entrenamiento comercial' y tiene un máster: canal doble (clínicas y alumnos).</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Por llamar</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr"/>
+      <c r="J5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>AF Dental Consulting</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Sin confirmar</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Formación comercial in company para clínicas: presentación de tratamientos, gestión de objeciones y seguimiento de presupuestos, para coordinadores de tratamiento.</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr"/>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>https://afdentalconsulting.com/formacion-comercial-clinicas-dentales</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Es exactamente lo que practica Zestiqa.</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>Por llamar</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr"/>
+      <c r="J6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Primerared S.L.</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Valencia</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Consultoría de gestión integral de clínicas dentales. Buscaba consultor/a en Valencia para presentar planes de tratamiento y hacer seguimiento de presupuestos pendientes (oferta en InfoJobs).</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>(buscar web)</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Está en Valencia y trabaja el seguimiento de presupuestos.</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Por llamar</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Enfoque Dental</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Sin confirmar</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Estrategia, formación, marketing y acompañamiento; protocolos para subir la aceptación y el presupuesto medio. Máster online de gestión.</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr"/>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>https://enfoquedental.com/</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Trabaja la aceptación de presupuestos.</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Por llamar</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr"/>
+      <c r="J8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>OdontoSupport</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Madrid (sin confirmar)</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Consultoría, formación, marketing y nuevas aperturas; aumentar el porcentaje de aceptación.</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>María Peidro, fundadora (web propia)</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>https://www.odontosupport.es/</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Trabaja la aceptación; formación en técnicas de venta.</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Por llamar</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Talent Clinics (Global Talent Clinics)</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Sin confirmar</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Consultoría de recursos humanos para clínicas: roles, liderazgo, formación y seguimiento del equipo.</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Cofundada por Fran Caro</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>https://talentclinics.com/consultoria-recursos-humanos/</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Forma equipos de clínica; puede entrar junto con Fran Caro.</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Por llamar</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr"/>
+      <c r="J10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>AESINERGY</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Sin confirmar</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Gestión dental, análisis económico, coaching de equipo y formación; cursos bonificables de coordinación.</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr"/>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>https://aesinergy.es/</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Ya da cursos de coordinación bonificables.</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>Por llamar</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr"/>
+      <c r="J11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>DND Consultoría</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Sin confirmar</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Consultoría y coaching dental desde hace más de 10 años; curso Experto en Gestión y Dirección de Clínica Dental.</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr"/>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>https://www.dndconsultoria.es/es/consultoria-y-coaching-dental</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Más centrada en gestión que en comercial.</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Por llamar</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr"/>
+      <c r="J12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Gestión Dental Integral (GDI)</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Sin confirmar</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Formaciones y consultoría para clínicas desde hace 15 años.</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr"/>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>(buscar web)</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Confirmar si forma a coordinadoras.</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>Por llamar</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr"/>
+      <c r="J13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Eusklinic</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>País Vasco (sin confirmar)</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Consultoría dental de gestión y marketing para clínicas.</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr"/>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>https://eusklinic.com/</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Lejos; solo por videollamada.</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>Por llamar</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr"/>
+      <c r="J14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Deac by Proclinic</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Sin confirmar</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Cursos de coordinación de la clínica dental (Proclinic es un gran distribuidor dental).</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr"/>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>https://www.deacbyproclinic.com/cursos/coordinacion-de-la-clinica-dental/</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Canal grande; difícil de entrada, pero llega a muchas clínicas.</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>Por llamar</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr"/>
+      <c r="J15" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J15"/>
+  <dataValidations count="1">
+    <dataValidation sqref="H2:H15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Por llamar,Llamado sin respuesta,Volver a llamar,Cita agendada,Visitado,No interesa,Descartado"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:P49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3540,7 +4170,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5409,7 +6039,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7235,7 +7865,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>